<commit_message>
:sparkles: feat: UI do simulador
</commit_message>
<xml_diff>
--- a/tabelas_comparativas.xlsx
+++ b/tabelas_comparativas.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Tabelas Consolidadas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Histórico de Passos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.00000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +44,14 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +68,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8EEF0"/>
         <bgColor rgb="00E8EEF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00374151"/>
+        <bgColor rgb="00374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+        <bgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -112,6 +137,15 @@
     </xf>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -492,7 +526,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>EXEMPLO: COS(X) - X</t>
+          <t>EXEMPLO DE TESTE: COS(X) - X = 0</t>
         </is>
       </c>
     </row>
@@ -541,7 +575,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.042</v>
+        <v>0.0381</v>
       </c>
       <c r="F4" s="7" t="n">
         <v>1.075020766849732e-07</v>
@@ -565,7 +599,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.0119</v>
+        <v>0.011</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>5.870465491497612e-07</v>
@@ -589,7 +623,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.0092</v>
+        <v>0.0105</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>1.180977871051425e-09</v>
@@ -613,7 +647,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>3.52926228242012e-08</v>
@@ -627,7 +661,7 @@
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>PROBLEMA 1: RESFRIAMENTO</t>
+          <t>PROBLEMA 1: RESFRIAMENTO DE COMPONENTE ELETRÔNICO</t>
         </is>
       </c>
     </row>
@@ -676,7 +710,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.0257</v>
+        <v>0.0267</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>1.479877909105198e-07</v>
@@ -700,7 +734,7 @@
         <v>21</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0.0328</v>
+        <v>0.032</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>7.023267940553524e-07</v>
@@ -724,7 +758,7 @@
         <v>5</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>0.0077</v>
+        <v>0.0075</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>3.965681116824271e-10</v>
@@ -748,7 +782,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.0105</v>
+        <v>0.0106</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2.133759835487581e-10</v>
@@ -762,7 +796,7 @@
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>PROBLEMA 2: CIRCUITO RC</t>
+          <t>PROBLEMA 2: CARREGAMENTO DE CAPACITOR EM CIRCUITO RC</t>
         </is>
       </c>
     </row>
@@ -811,7 +845,7 @@
         <v>21</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.0228</v>
+        <v>0.0203</v>
       </c>
       <c r="F20" s="7" t="n">
         <v>6.182878182769969e-07</v>
@@ -835,7 +869,7 @@
         <v>25</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.038</v>
+        <v>0.0379</v>
       </c>
       <c r="F21" s="7" t="n">
         <v>8.124089330152628e-07</v>
@@ -859,7 +893,7 @@
         <v>5</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0077</v>
       </c>
       <c r="F22" s="7" t="n">
         <v>8.178832722194329e-09</v>
@@ -883,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.0191</v>
+        <v>0.0133</v>
       </c>
       <c r="F23" s="7" t="n">
         <v>5.550284676303363e-10</v>
@@ -902,4 +936,3302 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F192"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>EXEMPLO DE TESTE: COS(X) - X = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Método: Bissecção (20 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0.3775825618903728</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0.3775825618903728</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>[0.000000, 1.000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>-0.0183111311261791</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0.0183111311261791</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>[0.500000, 1.000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.1859631195052179</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.1859631195052179</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>[0.500000, 0.750000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.0853349461524715</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.0853349461524715</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>[0.625000, 0.750000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.03387937241806649</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0.03387937241806649</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>[0.687500, 0.750000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0.734375</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.007874725458501319</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>0.007874725458501319</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>[0.718750, 0.750000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0.7421875</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>-0.005195711743759213</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.005195711743759213</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>[0.734375, 0.750000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0.73828125</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>0.001345149751805108</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.001345149751805108</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>[0.734375, 0.742188]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0.740234375</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>-0.001923872780897673</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.001923872780897673</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>[0.738281, 0.742188]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.7392578125</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>-0.0002890091467900868</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.0002890091467900868</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>[0.738281, 0.740234]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>0.73876953125</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>0.0005281584336581657</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.0005281584336581657</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>[0.738281, 0.739258]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>0.739013671875</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.0001195966713218866</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.0001195966713218866</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>[0.738770, 0.739258]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>0.7391357421875</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>-8.470073137478717e-05</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>8.470073137478717e-05</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>[0.739014, 0.739258]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>0.73907470703125</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>1.744934663994169e-05</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>1.744934663994169e-05</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>[0.739014, 0.739136]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>0.739105224609375</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>-3.362534821038654e-05</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>3.362534821038654e-05</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>[0.739075, 0.739136]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>0.7390899658203125</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>-8.087914744714375e-06</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>8.087914744714375e-06</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>[0.739075, 0.739105]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>0.7390823364257812</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>4.680737457851691e-06</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>4.680737457851691e-06</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>[0.739075, 0.739090]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>0.7390861511230469</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>-1.703583265899589e-06</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>1.703583265899589e-06</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>[0.739082, 0.739090]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="B23" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>0.7390842437744141</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>1.488578440400623e-06</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>1.488578440400623e-06</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>[0.739082, 0.739086]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0.7390851974487305</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>-1.075020766849732e-07</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>1.075020766849732e-07</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>[0.739084, 0.739086]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Método: Falsa Posição (5 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0.6850733573260451</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0.08929927648185998</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>0.08929927648185998</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0.736298997613654</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>0.004660039038142605</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0.004660039038142605</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.6851, 1.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0.7389453559657132</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.000233925665770629</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.000233925665770629</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.7363, 1.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0.7390781308800257</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>1.171917419451329e-05</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>1.171917419451329e-05</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.7389, 1.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="B32" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0.7390847824489231</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>5.870465491497612e-07</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>5.870465491497612e-07</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.7391, 1.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Método: Newton-Raphson (3 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="B36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>0.3775825618903728</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>0.02710331185746728</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -1.479426</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="B37" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0.7552224171056364</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>-0.02710331185746728</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>9.461538061772412e-05</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -1.685451</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>0.7391416661498792</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>-9.461538061772412e-05</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>1.180977871051425e-09</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -1.673654</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Método: Secante (4 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="B42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>0.6850733573260451</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>0.08929927648185998</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>0.08929927648185998</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.0000, xd=1.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>0.736298997613654</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>0.004660039038142605</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>0.004660039038142605</v>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.0000, xd=0.6851</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>0.7391193619116293</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>-5.728599110610411e-05</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>5.728599110610411e-05</v>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.6851, xd=0.7363</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="B45" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>0.7390851121274639</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>3.52926228242012e-08</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>3.52926228242012e-08</v>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.7363, xd=0.7391</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>PROBLEMA 1: RESFRIAMENTO DE COMPONENTE ELETRÔNICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Método: Bissecção (25 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F51" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="B52" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>12.51298974669132</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>12.51298974669132</v>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>[0.000000, 10.000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="B53" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>-0.7812779377485271</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>0.7812779377485271</v>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>[5.000000, 10.000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="B54" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>5.244506400911909</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>5.244506400911909</v>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>[5.000000, 7.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="B55" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>6.875</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>2.090488259755226</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>2.090488259755226</v>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>[6.250000, 7.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="B56" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>7.1875</v>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>0.620957811664411</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>0.620957811664411</v>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>[6.875000, 7.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="B57" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" s="4" t="n">
+        <v>7.34375</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>-0.08837591204799367</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>0.08837591204799367</v>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>[7.187500, 7.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="B58" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>7.265625</v>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>0.2642128474464585</v>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>0.2642128474464585</v>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>[7.187500, 7.343750]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="B59" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C59" s="4" t="n">
+        <v>7.3046875</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>0.08740198173624947</v>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>0.08740198173624947</v>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>[7.265625, 7.343750]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="B60" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>7.32421875</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>-0.0006157086383353771</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>0.0006157086383353771</v>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>[7.304688, 7.343750]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="B61" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C61" s="4" t="n">
+        <v>7.314453125</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>0.04336090351380761</v>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>0.04336090351380761</v>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>[7.304688, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="B62" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C62" s="4" t="n">
+        <v>7.3193359375</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>0.02136454507991203</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>0.02136454507991203</v>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>[7.314453, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="B63" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C63" s="4" t="n">
+        <v>7.32177734375</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>0.01037240586848043</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>0.01037240586848043</v>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>[7.319336, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="B64" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C64" s="4" t="n">
+        <v>7.322998046875</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>0.004877845619105869</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>0.004877845619105869</v>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>[7.321777, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="B65" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C65" s="4" t="n">
+        <v>7.3236083984375</v>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>0.002130942752906151</v>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>0.002130942752906151</v>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>[7.322998, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="B66" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C66" s="4" t="n">
+        <v>7.32391357421875</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>0.0007575856243562384</v>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>0.0007575856243562384</v>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>[7.323608, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="B67" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C67" s="4" t="n">
+        <v>7.324066162109375</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>7.093063495489105e-05</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>7.093063495489105e-05</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>[7.323914, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="B68" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C68" s="4" t="n">
+        <v>7.324142456054688</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>-0.0002723909661810353</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <v>0.0002723909661810353</v>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>[7.324066, 7.324219]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="B69" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C69" s="4" t="n">
+        <v>7.324104309082031</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>-0.0001007306567402111</v>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>0.0001007306567402111</v>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>[7.324066, 7.324142]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="B70" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C70" s="4" t="n">
+        <v>7.324085235595703</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>-1.490013367799747e-05</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>1.490013367799747e-05</v>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>[7.324066, 7.324104]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="B71" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>7.324075698852539</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>2.801521994655332e-05</v>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>2.801521994655332e-05</v>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>[7.324066, 7.324085]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="B72" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C72" s="4" t="n">
+        <v>7.324080467224121</v>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>6.557535463969089e-06</v>
+      </c>
+      <c r="E72" s="7" t="n">
+        <v>6.557535463969089e-06</v>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>[7.324076, 7.324085]</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="B73" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C73" s="4" t="n">
+        <v>7.324082851409912</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>-4.171301021926865e-06</v>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>4.171301021926865e-06</v>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>[7.324080, 7.324085]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="B74" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="C74" s="4" t="n">
+        <v>7.324081659317017</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>1.193116737852051e-06</v>
+      </c>
+      <c r="E74" s="7" t="n">
+        <v>1.193116737852051e-06</v>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>[7.324080, 7.324083]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="B75" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C75" s="4" t="n">
+        <v>7.324082255363464</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>-1.489092262829672e-06</v>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>1.489092262829672e-06</v>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>[7.324082, 7.324083]</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="B76" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C76" s="4" t="n">
+        <v>7.32408195734024</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>-1.479877909105198e-07</v>
+      </c>
+      <c r="E76" s="7" t="n">
+        <v>1.479877909105198e-07</v>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>[7.324082, 7.324082]</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>Método: Falsa Posição (21 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="B80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>8.581446111925787</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>-5.156584352718852</v>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>5.156584352718852</v>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 10.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="B81" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" s="4" t="n">
+        <v>7.902298314599451</v>
+      </c>
+      <c r="D81" s="7" t="n">
+        <v>-2.492328672347156</v>
+      </c>
+      <c r="E81" s="7" t="n">
+        <v>2.492328672347156</v>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 8.5814]</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="B82" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C82" s="4" t="n">
+        <v>7.587137636715609</v>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>-1.160700445699796</v>
+      </c>
+      <c r="E82" s="7" t="n">
+        <v>1.160700445699796</v>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.9023]</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="B83" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C83" s="4" t="n">
+        <v>7.443149847623166</v>
+      </c>
+      <c r="D83" s="7" t="n">
+        <v>-0.5310492183180386</v>
+      </c>
+      <c r="E83" s="7" t="n">
+        <v>0.5310492183180386</v>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.5871]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="B84" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C84" s="4" t="n">
+        <v>7.37784982458626</v>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>-0.240982460262309</v>
+      </c>
+      <c r="E84" s="7" t="n">
+        <v>0.240982460262309</v>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.4431]</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="B85" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C85" s="4" t="n">
+        <v>7.348336155825173</v>
+      </c>
+      <c r="D85" s="7" t="n">
+        <v>-0.1089457413613033</v>
+      </c>
+      <c r="E85" s="7" t="n">
+        <v>0.1089457413613033</v>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3778]</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="B86" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C86" s="4" t="n">
+        <v>7.335017507154921</v>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>-0.0491697836111058</v>
+      </c>
+      <c r="E86" s="7" t="n">
+        <v>0.0491697836111058</v>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3483]</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="B87" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C87" s="4" t="n">
+        <v>7.329011408737406</v>
+      </c>
+      <c r="D87" s="7" t="n">
+        <v>-0.02217448010837586</v>
+      </c>
+      <c r="E87" s="7" t="n">
+        <v>0.02217448010837586</v>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3350]</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="B88" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C88" s="4" t="n">
+        <v>7.326303792442182</v>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>-0.009996739996253723</v>
+      </c>
+      <c r="E88" s="7" t="n">
+        <v>0.009996739996253723</v>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3290]</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="B89" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C89" s="4" t="n">
+        <v>7.325083343214965</v>
+      </c>
+      <c r="D89" s="7" t="n">
+        <v>-0.004506045982651585</v>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>0.004506045982651585</v>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3263]</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="B90" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C90" s="4" t="n">
+        <v>7.324533265153394</v>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>-0.002030964396936952</v>
+      </c>
+      <c r="E90" s="7" t="n">
+        <v>0.002030964396936952</v>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3251]</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="B91" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C91" s="4" t="n">
+        <v>7.324285342440669</v>
+      </c>
+      <c r="D91" s="7" t="n">
+        <v>-0.000915366974489018</v>
+      </c>
+      <c r="E91" s="7" t="n">
+        <v>0.000915366974489018</v>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3245]</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="B92" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C92" s="4" t="n">
+        <v>7.324173603996794</v>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>-0.0004125551055551568</v>
+      </c>
+      <c r="E92" s="7" t="n">
+        <v>0.0004125551055551568</v>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3243]</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="B93" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C93" s="4" t="n">
+        <v>7.324123243922827</v>
+      </c>
+      <c r="D93" s="7" t="n">
+        <v>-0.0001859370332226717</v>
+      </c>
+      <c r="E93" s="7" t="n">
+        <v>0.0001859370332226717</v>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3242]</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="B94" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C94" s="4" t="n">
+        <v>7.324100546897382</v>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>-8.380087788850688e-05</v>
+      </c>
+      <c r="E94" s="7" t="n">
+        <v>8.380087788850688e-05</v>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="B95" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C95" s="4" t="n">
+        <v>7.32409031747741</v>
+      </c>
+      <c r="D95" s="7" t="n">
+        <v>-3.776858127935157e-05</v>
+      </c>
+      <c r="E95" s="7" t="n">
+        <v>3.776858127935157e-05</v>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="B96" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C96" s="4" t="n">
+        <v>7.324085707138638</v>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>-1.702207574538761e-05</v>
+      </c>
+      <c r="E96" s="7" t="n">
+        <v>1.702207574538761e-05</v>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="B97" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C97" s="4" t="n">
+        <v>7.324083629286866</v>
+      </c>
+      <c r="D97" s="7" t="n">
+        <v>-7.671746622861519e-06</v>
+      </c>
+      <c r="E97" s="7" t="n">
+        <v>7.671746622861519e-06</v>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="B98" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C98" s="4" t="n">
+        <v>7.324082692811755</v>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>-3.457609409451834e-06</v>
+      </c>
+      <c r="E98" s="7" t="n">
+        <v>3.457609409451834e-06</v>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="B99" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C99" s="4" t="n">
+        <v>7.324082270748159</v>
+      </c>
+      <c r="D99" s="7" t="n">
+        <v>-1.558323376116277e-06</v>
+      </c>
+      <c r="E99" s="7" t="n">
+        <v>1.558323376116277e-06</v>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="B100" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C100" s="4" t="n">
+        <v>7.324082080526686</v>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>-7.023267940553524e-07</v>
+      </c>
+      <c r="E100" s="7" t="n">
+        <v>7.023267940553524e-07</v>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 7.3241]</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>Método: Newton-Raphson (5 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="B104" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>16.20754071293328</v>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -13.500000</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="B105" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C105" s="4" t="n">
+        <v>4.444444444444445</v>
+      </c>
+      <c r="D105" s="7" t="n">
+        <v>16.20754071293328</v>
+      </c>
+      <c r="E105" s="7" t="n">
+        <v>2.537318236091615</v>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -6.931131</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="B106" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C106" s="4" t="n">
+        <v>6.782813242100721</v>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>2.537318236091615</v>
+      </c>
+      <c r="E106" s="7" t="n">
+        <v>0.09641002977141255</v>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -4.880598</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="B107" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C107" s="4" t="n">
+        <v>7.302691825348991</v>
+      </c>
+      <c r="D107" s="7" t="n">
+        <v>0.09641002977141255</v>
+      </c>
+      <c r="E107" s="7" t="n">
+        <v>0.0001542538922478798</v>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -4.514462</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="B108" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C108" s="4" t="n">
+        <v>7.324047645899469</v>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>0.0001542538922478798</v>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>3.965681116824271e-10</v>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = -4.500023</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>Método: Secante (6 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="B112" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" s="4" t="n">
+        <v>8.581446111925787</v>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>-5.156584352718852</v>
+      </c>
+      <c r="E112" s="7" t="n">
+        <v>5.156584352718852</v>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.0000, xd=10.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="B113" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C113" s="4" t="n">
+        <v>7.04525296931102</v>
+      </c>
+      <c r="D113" s="7" t="n">
+        <v>1.281339102206161</v>
+      </c>
+      <c r="E113" s="7" t="n">
+        <v>1.281339102206161</v>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>xe=10.0000, xd=8.5814</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="B114" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C114" s="4" t="n">
+        <v>7.351001298870212</v>
+      </c>
+      <c r="D114" s="7" t="n">
+        <v>-0.1208929434319401</v>
+      </c>
+      <c r="E114" s="7" t="n">
+        <v>0.1208929434319401</v>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>xe=8.5814, xd=7.0453</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="B115" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C115" s="4" t="n">
+        <v>7.324641313998386</v>
+      </c>
+      <c r="D115" s="7" t="n">
+        <v>-0.002517147343027659</v>
+      </c>
+      <c r="E115" s="7" t="n">
+        <v>0.002517147343027659</v>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>xe=7.0453, xd=7.3510</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="B116" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C116" s="4" t="n">
+        <v>7.324080794296939</v>
+      </c>
+      <c r="D116" s="7" t="n">
+        <v>5.08570749957471e-06</v>
+      </c>
+      <c r="E116" s="7" t="n">
+        <v>5.08570749957471e-06</v>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>xe=7.3510, xd=7.3246</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="B117" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C117" s="4" t="n">
+        <v>7.32408192450148</v>
+      </c>
+      <c r="D117" s="7" t="n">
+        <v>-2.133759835487581e-10</v>
+      </c>
+      <c r="E117" s="7" t="n">
+        <v>2.133759835487581e-10</v>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>xe=7.3246, xd=7.3241</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="26" customHeight="1">
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>PROBLEMA 2: CARREGAMENTO DE CAPACITOR EM CIRCUITO RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>Método: Bissecção (21 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="B124" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D124" s="7" t="n">
+        <v>0.08434919925785112</v>
+      </c>
+      <c r="E124" s="7" t="n">
+        <v>0.08434919925785112</v>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>[0.000000, 3.000000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="18" customHeight="1">
+      <c r="B125" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D125" s="7" t="n">
+        <v>-1.161832763705073</v>
+      </c>
+      <c r="E125" s="7" t="n">
+        <v>1.161832763705073</v>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>[0.000000, 1.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="18" customHeight="1">
+      <c r="B126" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C126" s="4" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="D126" s="7" t="n">
+        <v>-0.4232623367917485</v>
+      </c>
+      <c r="E126" s="7" t="n">
+        <v>0.4232623367917485</v>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>[0.750000, 1.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="18" customHeight="1">
+      <c r="B127" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C127" s="4" t="n">
+        <v>1.3125</v>
+      </c>
+      <c r="D127" s="7" t="n">
+        <v>-0.1457317436459191</v>
+      </c>
+      <c r="E127" s="7" t="n">
+        <v>0.1457317436459191</v>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>[1.125000, 1.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="B128" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C128" s="4" t="n">
+        <v>1.40625</v>
+      </c>
+      <c r="D128" s="7" t="n">
+        <v>-0.02530269622762926</v>
+      </c>
+      <c r="E128" s="7" t="n">
+        <v>0.02530269622762926</v>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>[1.312500, 1.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="B129" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C129" s="4" t="n">
+        <v>1.453125</v>
+      </c>
+      <c r="D129" s="7" t="n">
+        <v>0.03080799942957668</v>
+      </c>
+      <c r="E129" s="7" t="n">
+        <v>0.03080799942957668</v>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>[1.406250, 1.500000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="B130" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C130" s="4" t="n">
+        <v>1.4296875</v>
+      </c>
+      <c r="D130" s="7" t="n">
+        <v>0.00308141015910568</v>
+      </c>
+      <c r="E130" s="7" t="n">
+        <v>0.00308141015910568</v>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>[1.406250, 1.453125]</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="18" customHeight="1">
+      <c r="B131" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C131" s="4" t="n">
+        <v>1.41796875</v>
+      </c>
+      <c r="D131" s="7" t="n">
+        <v>-0.01102748742422044</v>
+      </c>
+      <c r="E131" s="7" t="n">
+        <v>0.01102748742422044</v>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>[1.406250, 1.429688]</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="18" customHeight="1">
+      <c r="B132" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C132" s="4" t="n">
+        <v>1.423828125</v>
+      </c>
+      <c r="D132" s="7" t="n">
+        <v>-0.003952371361242601</v>
+      </c>
+      <c r="E132" s="7" t="n">
+        <v>0.003952371361242601</v>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>[1.417969, 1.429688]</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="B133" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C133" s="4" t="n">
+        <v>1.4267578125</v>
+      </c>
+      <c r="D133" s="7" t="n">
+        <v>-0.0004303289093039453</v>
+      </c>
+      <c r="E133" s="7" t="n">
+        <v>0.0004303289093039453</v>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>[1.423828, 1.429688]</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="18" customHeight="1">
+      <c r="B134" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C134" s="4" t="n">
+        <v>1.42822265625</v>
+      </c>
+      <c r="D134" s="7" t="n">
+        <v>0.001326826661927072</v>
+      </c>
+      <c r="E134" s="7" t="n">
+        <v>0.001326826661927072</v>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>[1.426758, 1.429688]</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="B135" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C135" s="4" t="n">
+        <v>1.427490234375</v>
+      </c>
+      <c r="D135" s="7" t="n">
+        <v>0.0004485706210917151</v>
+      </c>
+      <c r="E135" s="7" t="n">
+        <v>0.0004485706210917151</v>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>[1.426758, 1.428223]</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="B136" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C136" s="4" t="n">
+        <v>1.4271240234375</v>
+      </c>
+      <c r="D136" s="7" t="n">
+        <v>9.20132154824671e-06</v>
+      </c>
+      <c r="E136" s="7" t="n">
+        <v>9.20132154824671e-06</v>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>[1.426758, 1.427490]</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="B137" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C137" s="4" t="n">
+        <v>1.42694091796875</v>
+      </c>
+      <c r="D137" s="7" t="n">
+        <v>-0.0002105436737807054</v>
+      </c>
+      <c r="E137" s="7" t="n">
+        <v>0.0002105436737807054</v>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>[1.426758, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="18" customHeight="1">
+      <c r="B138" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C138" s="4" t="n">
+        <v>1.427032470703125</v>
+      </c>
+      <c r="D138" s="7" t="n">
+        <v>-0.0001006661465523528</v>
+      </c>
+      <c r="E138" s="7" t="n">
+        <v>0.0001006661465523528</v>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>[1.426941, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="18" customHeight="1">
+      <c r="B139" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C139" s="4" t="n">
+        <v>1.427078247070312</v>
+      </c>
+      <c r="D139" s="7" t="n">
+        <v>-4.573115516848247e-05</v>
+      </c>
+      <c r="E139" s="7" t="n">
+        <v>4.573115516848247e-05</v>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>[1.427032, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="B140" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C140" s="4" t="n">
+        <v>1.427101135253906</v>
+      </c>
+      <c r="D140" s="7" t="n">
+        <v>-1.826460248421924e-05</v>
+      </c>
+      <c r="E140" s="7" t="n">
+        <v>1.826460248421924e-05</v>
+      </c>
+      <c r="F140" s="3" t="inlineStr">
+        <is>
+          <t>[1.427078, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="B141" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C141" s="4" t="n">
+        <v>1.427112579345703</v>
+      </c>
+      <c r="D141" s="7" t="n">
+        <v>-4.531561887066715e-06</v>
+      </c>
+      <c r="E141" s="7" t="n">
+        <v>4.531561887066715e-06</v>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>[1.427101, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="B142" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C142" s="4" t="n">
+        <v>1.427118301391602</v>
+      </c>
+      <c r="D142" s="7" t="n">
+        <v>2.334899475542329e-06</v>
+      </c>
+      <c r="E142" s="7" t="n">
+        <v>2.334899475542329e-06</v>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>[1.427113, 1.427124]</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="B143" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C143" s="4" t="n">
+        <v>1.427115440368652</v>
+      </c>
+      <c r="D143" s="7" t="n">
+        <v>-1.098326294801666e-06</v>
+      </c>
+      <c r="E143" s="7" t="n">
+        <v>1.098326294801666e-06</v>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>[1.427113, 1.427118]</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="B144" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C144" s="4" t="n">
+        <v>1.427116870880127</v>
+      </c>
+      <c r="D144" s="7" t="n">
+        <v>6.182878182769969e-07</v>
+      </c>
+      <c r="E144" s="7" t="n">
+        <v>6.182878182769969e-07</v>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>[1.427115, 1.427118]</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="22" customHeight="1">
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>Método: Falsa Posição (25 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C147" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="B148" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" s="4" t="n">
+        <v>2.399462188000063</v>
+      </c>
+      <c r="D148" s="7" t="n">
+        <v>0.7461662219231844</v>
+      </c>
+      <c r="E148" s="7" t="n">
+        <v>0.7461662219231844</v>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 3.0000]</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="B149" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C149" s="4" t="n">
+        <v>2.005636369042184</v>
+      </c>
+      <c r="D149" s="7" t="n">
+        <v>0.5271268534363909</v>
+      </c>
+      <c r="E149" s="7" t="n">
+        <v>0.5271268534363909</v>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 2.3995]</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="B150" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C150" s="4" t="n">
+        <v>1.761311479996882</v>
+      </c>
+      <c r="D150" s="7" t="n">
+        <v>0.3409031084111787</v>
+      </c>
+      <c r="E150" s="7" t="n">
+        <v>0.3409031084111787</v>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 2.0056]</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="B151" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C151" s="4" t="n">
+        <v>1.616310125777413</v>
+      </c>
+      <c r="D151" s="7" t="n">
+        <v>0.2068486536850864</v>
+      </c>
+      <c r="E151" s="7" t="n">
+        <v>0.2068486536850864</v>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.7613]</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="18" customHeight="1">
+      <c r="B152" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C152" s="4" t="n">
+        <v>1.532870095381669</v>
+      </c>
+      <c r="D152" s="7" t="n">
+        <v>0.1204245985237389</v>
+      </c>
+      <c r="E152" s="7" t="n">
+        <v>0.1204245985237389</v>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.6163]</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="18" customHeight="1">
+      <c r="B153" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C153" s="4" t="n">
+        <v>1.485784566458375</v>
+      </c>
+      <c r="D153" s="7" t="n">
+        <v>0.06837647884929332</v>
+      </c>
+      <c r="E153" s="7" t="n">
+        <v>0.06837647884929332</v>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.5329]</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="18" customHeight="1">
+      <c r="B154" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C154" s="4" t="n">
+        <v>1.459522200957365</v>
+      </c>
+      <c r="D154" s="7" t="n">
+        <v>0.03826368243727352</v>
+      </c>
+      <c r="E154" s="7" t="n">
+        <v>0.03826368243727352</v>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4858]</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="B155" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C155" s="4" t="n">
+        <v>1.444972212048808</v>
+      </c>
+      <c r="D155" s="7" t="n">
+        <v>0.02123686226324217</v>
+      </c>
+      <c r="E155" s="7" t="n">
+        <v>0.02123686226324217</v>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4595]</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="18" customHeight="1">
+      <c r="B156" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C156" s="4" t="n">
+        <v>1.436941651016452</v>
+      </c>
+      <c r="D156" s="7" t="n">
+        <v>0.01173262182876478</v>
+      </c>
+      <c r="E156" s="7" t="n">
+        <v>0.01173262182876478</v>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4450]</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="B157" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C157" s="4" t="n">
+        <v>1.432518703592273</v>
+      </c>
+      <c r="D157" s="7" t="n">
+        <v>0.006465337815869443</v>
+      </c>
+      <c r="E157" s="7" t="n">
+        <v>0.006465337815869443</v>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4369]</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="B158" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C158" s="4" t="n">
+        <v>1.430085549333842</v>
+      </c>
+      <c r="D158" s="7" t="n">
+        <v>0.003557747997185778</v>
+      </c>
+      <c r="E158" s="7" t="n">
+        <v>0.003557747997185778</v>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4325]</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="B159" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C159" s="4" t="n">
+        <v>1.428747884879654</v>
+      </c>
+      <c r="D159" s="7" t="n">
+        <v>0.001956238823050072</v>
+      </c>
+      <c r="E159" s="7" t="n">
+        <v>0.001956238823050072</v>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4301]</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="B160" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C160" s="4" t="n">
+        <v>1.428012744361146</v>
+      </c>
+      <c r="D160" s="7" t="n">
+        <v>0.001075184501576842</v>
+      </c>
+      <c r="E160" s="7" t="n">
+        <v>0.001075184501576842</v>
+      </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4287]</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="18" customHeight="1">
+      <c r="B161" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C161" s="4" t="n">
+        <v>1.427608812027197</v>
+      </c>
+      <c r="D161" s="7" t="n">
+        <v>0.0005908021803686658</v>
+      </c>
+      <c r="E161" s="7" t="n">
+        <v>0.0005908021803686658</v>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4280]</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="18" customHeight="1">
+      <c r="B162" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C162" s="4" t="n">
+        <v>1.42738689010959</v>
+      </c>
+      <c r="D162" s="7" t="n">
+        <v>0.0003245974539538565</v>
+      </c>
+      <c r="E162" s="7" t="n">
+        <v>0.0003245974539538565</v>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4276]</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="B163" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C163" s="4" t="n">
+        <v>1.427264972589533</v>
+      </c>
+      <c r="D163" s="7" t="n">
+        <v>0.000178327087722252</v>
+      </c>
+      <c r="E163" s="7" t="n">
+        <v>0.000178327087722252</v>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4274]</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="18" customHeight="1">
+      <c r="B164" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C164" s="4" t="n">
+        <v>1.427197996783646</v>
+      </c>
+      <c r="D164" s="7" t="n">
+        <v>9.796537314343823e-05</v>
+      </c>
+      <c r="E164" s="7" t="n">
+        <v>9.796537314343823e-05</v>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4273]</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="18" customHeight="1">
+      <c r="B165" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C165" s="4" t="n">
+        <v>1.427161204052096</v>
+      </c>
+      <c r="D165" s="7" t="n">
+        <v>5.381688752992275e-05</v>
+      </c>
+      <c r="E165" s="7" t="n">
+        <v>5.381688752992275e-05</v>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4272]</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="B166" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C166" s="4" t="n">
+        <v>1.427140992397812</v>
+      </c>
+      <c r="D166" s="7" t="n">
+        <v>2.956374502049997e-05</v>
+      </c>
+      <c r="E166" s="7" t="n">
+        <v>2.956374502049997e-05</v>
+      </c>
+      <c r="F166" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4272]</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="B167" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C167" s="4" t="n">
+        <v>1.427129889423032</v>
+      </c>
+      <c r="D167" s="7" t="n">
+        <v>1.624042956693827e-05</v>
+      </c>
+      <c r="E167" s="7" t="n">
+        <v>1.624042956693827e-05</v>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="B168" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C168" s="4" t="n">
+        <v>1.427123790185296</v>
+      </c>
+      <c r="D168" s="7" t="n">
+        <v>8.921421017049624e-06</v>
+      </c>
+      <c r="E168" s="7" t="n">
+        <v>8.921421017049624e-06</v>
+      </c>
+      <c r="F168" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="B169" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C169" s="4" t="n">
+        <v>1.427120439674169</v>
+      </c>
+      <c r="D169" s="7" t="n">
+        <v>4.900830820275814e-06</v>
+      </c>
+      <c r="E169" s="7" t="n">
+        <v>4.900830820275814e-06</v>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="B170" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="C170" s="4" t="n">
+        <v>1.42711859913027</v>
+      </c>
+      <c r="D170" s="7" t="n">
+        <v>2.692185129493652e-06</v>
+      </c>
+      <c r="E170" s="7" t="n">
+        <v>2.692185129493652e-06</v>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="B171" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C171" s="4" t="n">
+        <v>1.427117588060599</v>
+      </c>
+      <c r="D171" s="7" t="n">
+        <v>1.478903633334028e-06</v>
+      </c>
+      <c r="E171" s="7" t="n">
+        <v>1.478903633334028e-06</v>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="B172" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C172" s="4" t="n">
+        <v>1.427117032647819</v>
+      </c>
+      <c r="D172" s="7" t="n">
+        <v>8.124089330152628e-07</v>
+      </c>
+      <c r="E172" s="7" t="n">
+        <v>8.124089330152628e-07</v>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>Secante entre [0.0000, 1.4271]</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="22" customHeight="1">
+      <c r="B174" s="9" t="inlineStr">
+        <is>
+          <t>Método: Newton-Raphson (5 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="20" customHeight="1">
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D175" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F175" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="18" customHeight="1">
+      <c r="B176" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C176" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" s="7" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="E176" s="7" t="n">
+        <v>1.138332135049546</v>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = 5.000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="18" customHeight="1">
+      <c r="B177" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C177" s="4" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="D177" s="7" t="n">
+        <v>-1.138332135049546</v>
+      </c>
+      <c r="E177" s="7" t="n">
+        <v>0.2370957048813707</v>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = 2.338332</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="18" customHeight="1">
+      <c r="B178" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C178" s="4" t="n">
+        <v>1.246813707080763</v>
+      </c>
+      <c r="D178" s="7" t="n">
+        <v>-0.2370957048813707</v>
+      </c>
+      <c r="E178" s="7" t="n">
+        <v>0.01852567114736914</v>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = 1.437096</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="18" customHeight="1">
+      <c r="B179" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C179" s="4" t="n">
+        <v>1.411796250745761</v>
+      </c>
+      <c r="D179" s="7" t="n">
+        <v>-0.01852567114736914</v>
+      </c>
+      <c r="E179" s="7" t="n">
+        <v>0.000140115150847997</v>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = 1.218526</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="18" customHeight="1">
+      <c r="B180" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C180" s="4" t="n">
+        <v>1.426999599830664</v>
+      </c>
+      <c r="D180" s="7" t="n">
+        <v>-0.000140115150847997</v>
+      </c>
+      <c r="E180" s="7" t="n">
+        <v>8.178832722194329e-09</v>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>f'(x) = 1.200140</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="22" customHeight="1">
+      <c r="B182" s="9" t="inlineStr">
+        <is>
+          <t>Método: Secante (9 iterações)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>Iteração</t>
+        </is>
+      </c>
+      <c r="C183" s="10" t="inlineStr">
+        <is>
+          <t>Estimativa (x)</t>
+        </is>
+      </c>
+      <c r="D183" s="10" t="inlineStr">
+        <is>
+          <t>f(x)</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="inlineStr">
+        <is>
+          <t>Precisão |f(x)|</t>
+        </is>
+      </c>
+      <c r="F183" s="10" t="inlineStr">
+        <is>
+          <t>Detalhes / Intervalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="18" customHeight="1">
+      <c r="B184" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C184" s="4" t="n">
+        <v>2.399462188000063</v>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>0.7461662219231844</v>
+      </c>
+      <c r="E184" s="7" t="n">
+        <v>0.7461662219231844</v>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.0000, xd=3.0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="18" customHeight="1">
+      <c r="B185" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C185" s="4" t="n">
+        <v>0.2125200203076823</v>
+      </c>
+      <c r="D185" s="7" t="n">
+        <v>-2.842720644285898</v>
+      </c>
+      <c r="E185" s="7" t="n">
+        <v>2.842720644285898</v>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>xe=3.0000, xd=2.3995</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="18" customHeight="1">
+      <c r="B186" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C186" s="4" t="n">
+        <v>1.944774582716142</v>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>0.4849027061866078</v>
+      </c>
+      <c r="E186" s="7" t="n">
+        <v>0.4849027061866078</v>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>xe=2.3995, xd=0.2125</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="18" customHeight="1">
+      <c r="B187" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C187" s="4" t="n">
+        <v>1.692349702659724</v>
+      </c>
+      <c r="D187" s="7" t="n">
+        <v>0.2795676652321166</v>
+      </c>
+      <c r="E187" s="7" t="n">
+        <v>0.2795676652321166</v>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>xe=0.2125, xd=1.9448</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="18" customHeight="1">
+      <c r="B188" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C188" s="4" t="n">
+        <v>1.348668302564401</v>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>-0.09792860104475576</v>
+      </c>
+      <c r="E188" s="7" t="n">
+        <v>0.09792860104475576</v>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.9448, xd=1.6923</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="18" customHeight="1">
+      <c r="B189" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C189" s="4" t="n">
+        <v>1.437824783629443</v>
+      </c>
+      <c r="D189" s="7" t="n">
+        <v>0.01278155626110422</v>
+      </c>
+      <c r="E189" s="7" t="n">
+        <v>0.01278155626110422</v>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.6923, xd=1.3487</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="18" customHeight="1">
+      <c r="B190" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C190" s="4" t="n">
+        <v>1.427531612645803</v>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>0.0004982049580792847</v>
+      </c>
+      <c r="E190" s="7" t="n">
+        <v>0.0004982049580792847</v>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.3487, xd=1.4378</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="18" customHeight="1">
+      <c r="B191" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C191" s="4" t="n">
+        <v>1.427114128142437</v>
+      </c>
+      <c r="D191" s="7" t="n">
+        <v>-2.673000226938171e-06</v>
+      </c>
+      <c r="E191" s="7" t="n">
+        <v>2.673000226938171e-06</v>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.4378, xd=1.4275</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="18" customHeight="1">
+      <c r="B192" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C192" s="4" t="n">
+        <v>1.427116356102669</v>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>5.550284676303363e-10</v>
+      </c>
+      <c r="E192" s="7" t="n">
+        <v>5.550284676303363e-10</v>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>xe=1.4275, xd=1.4271</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B110:F110"/>
+    <mergeCell ref="B182:F182"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B78:F78"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B174:F174"/>
+    <mergeCell ref="B146:F146"/>
+    <mergeCell ref="B121:F121"/>
+    <mergeCell ref="B122:F122"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B102:F102"/>
+    <mergeCell ref="B49:F49"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>